<commit_message>
Refactor report classes into separate files; update build config
Refactored internal report-related classes from Reports.cs into individual files under Transmittal.Reports.OpenXML for improved modularity and maintainability. Updated solution to use "Debug|x64" build configuration. Modified several Excel template files.
</commit_message>
<xml_diff>
--- a/source/Transmittal.Reports.OpenXML/Reports/MasterDocumentsList.xlsx
+++ b/source/Transmittal.Reports.OpenXML/Reports/MasterDocumentsList.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8cb514c15eb25f74/Transmittal Testing/Reports/Style3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{50C3F467-2AB6-4275-8A3C-BCC2AC95F285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A12B7B7-3F00-4178-9B90-75E8D97F1A1E}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{50C3F467-2AB6-4275-8A3C-BCC2AC95F285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84D5A009-37E3-4BE2-B316-2A84BD981F07}"/>
   <bookViews>
-    <workbookView xWindow="32475" yWindow="1935" windowWidth="24975" windowHeight="19290" xr2:uid="{CA3D9014-5C30-45DF-BF22-4326D1D6B854}"/>
+    <workbookView xWindow="3900" yWindow="1650" windowWidth="35145" windowHeight="19230" xr2:uid="{CA3D9014-5C30-45DF-BF22-4326D1D6B854}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Documents" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="MasterDocumentListData">'Master Documents'!$A$8:$D$8</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>{{ReportTitle}}</t>
   </si>
@@ -57,6 +60,21 @@
   </si>
   <si>
     <t>Document ID</t>
+  </si>
+  <si>
+    <t>{{DrgStatus}}</t>
+  </si>
+  <si>
+    <t>{{DrgRev}}</t>
+  </si>
+  <si>
+    <t>{{DrgName}}</t>
+  </si>
+  <si>
+    <t>Document ID format: &lt;Project&gt;-&lt;Originator&gt;-&lt;Volume&gt;-&lt;Level&gt;-&lt;Type&gt;-&lt;Role&gt;-&lt;DocNo&gt;</t>
+  </si>
+  <si>
+    <t>{{DrgProj}}-{{DrgOriginator}}-{{DrgVolume}}-{{DrgLevel}}-{{DrgType}}-{{DrgRole}}-{{DrgNumber}}</t>
   </si>
 </sst>
 </file>
@@ -108,10 +126,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -450,45 +471,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22515EDA-C0CF-49E9-867A-7E79AA4CF41E}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
     <col min="3" max="3" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>